<commit_message>
Rename minimize_haircut to calibrate_and_solve_ge
Added code/calibrate_and_solve_ge.m and update the file header to reflect calibration + V0-maximising GE solver pattern. Remove legacy solver scripts code/solve_ge_model.m and code/solve_ge_model_value_max.m (cleanup of duplicated/old implementations). This consolidates the calibration/solution entry point and clarifies the solver approach in the header comments.
</commit_message>
<xml_diff>
--- a/data/sri_lanka_CDS.xlsx
+++ b/data/sri_lanka_CDS.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/39cf3870e3a2584e/Documents/Oxford/Thesis/MPhil-Thesis/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="264" documentId="8_{587AD4E2-4611-4E04-BAB5-AEF13A89D962}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0BAC2CBF-F1CE-4AD6-B6E6-3A406E697279}"/>
+  <xr:revisionPtr revIDLastSave="269" documentId="8_{587AD4E2-4611-4E04-BAB5-AEF13A89D962}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0F9638B6-2D69-4910-A866-2016F4289EC6}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{04AEC5C9-B1EC-4CD4-951C-5C617ABD1667}"/>
+    <workbookView xWindow="3465" yWindow="3465" windowWidth="28800" windowHeight="15285" xr2:uid="{04AEC5C9-B1EC-4CD4-951C-5C617ABD1667}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -225,10 +225,10 @@
   <volType type="realTimeData">
     <main first="refinitivshim.rtdserver.rdp.historicalpricing">
       <tp t="s">
-        <v>Updated at 14:43:18</v>
+        <v>Not Signed In</v>
         <stp/>
-        <stp>8</stp>
-        <stp>61762718</stp>
+        <stp>1</stp>
+        <stp>102018343</stp>
         <tr r="A1" s="1"/>
       </tp>
     </main>
@@ -574,7 +574,7 @@
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" t="str">
         <f>_xll.RDP.HistoricalPricing("LKGV5YUSAC=R",C1:E1,"START:01-Jan-2015 END:01-Jan-2025 INTERVAL:P1D SOURCE:RFV",,"CH:Fd RH:Timestamp",B2)</f>
-        <v>Updated at 14:43:18</v>
+        <v>Not Signed In</v>
       </c>
       <c r="B1" t="s">
         <v>9</v>

</xml_diff>